<commit_message>
Add 4 Axis Bank offers to the batch 2 sheet - 33 offers, 10 issuers
Read from axis.bank.in/offers (verified by 301 redirect from axisbank.com).
All four valid to 15 Oct 2026. KFC (freebie, no discount value), SNITCH and
the Apple banner (headline only, no published value) are excluded and noted
in the README sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deployment_assets/offerlens_batch2_offers.xlsx
+++ b/deployment_assets/offerlens_batch2_offers.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2448,6 +2448,276 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Bata</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Axis Bank</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Rs 500 off at Bata with Axis Bank Credit and Debit Cards.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Minimum shopping of Rs 2,999. Valid on Credit and Debit Cards.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bata.in</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.axis.bank.in/offers</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>AJIO</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Axis Bank</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="n">
+        <v>1299</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Flat Rs 150 off on AJIO with Axis Bank Credit and Debit Cards.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Minimum order value Rs 1,299. Valid on Credit and Debit Cards.</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>ADNAJIO</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ajio.com</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.axis.bank.in/offers</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Urban Ladder</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Axis Bank</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Additional 10% off on Urban Ladder with Axis Bank Credit and Debit Cards.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Minimum order Rs 5,000. Stated as an additional discount, so it applies on top of any existing offer. No cap published by the issuer.</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>ULADN10</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.urbanladder.com</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.axis.bank.in/offers</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Yes Madam</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Axis Bank</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Health &amp; Beauty</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Rs 500 off on Yes Madam with Axis Bank Credit and Debit Cards.</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Minimum order not published by the issuer.</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>YMADN500</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.yesmadam.com</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.axis.bank.in/offers</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2459,7 +2729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -2478,7 +2748,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Built 30 July 2026. 29 offers across 9 issuers.</t>
+          <t>Built 30 July 2026. 33 offers across 10 issuers.</t>
         </is>
       </c>
     </row>
@@ -2662,6 +2932,20 @@
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Citibank - has exited Indian consumer banking; no such card exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Axis KFC (free fries) - a freebie, not a discount value; does not fit the schema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Axis SNITCH and the Apple banner - headline only, no value published.</t>
         </is>
       </c>
     </row>

</xml_diff>